<commit_message>
Segunda versão dos requisitos
</commit_message>
<xml_diff>
--- a/Requisitos.xlsx
+++ b/Requisitos.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
   <fileVersion appName="Calc"/>
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="170" uniqueCount="116">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="480" uniqueCount="206">
   <si>
     <t xml:space="preserve">N Requisito</t>
   </si>
@@ -36,10 +36,28 @@
     <t xml:space="preserve">Dependências</t>
   </si>
   <si>
+    <t xml:space="preserve">Prioridade</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Status</t>
+  </si>
+  <si>
     <t xml:space="preserve">RNE0</t>
   </si>
   <si>
-    <t xml:space="preserve">O cadastro deve obrigatoriamente ter : usuário, senha e e-mail</t>
+    <t xml:space="preserve">O cadastro deve obrigatoriamente ter: usuário, senha e e-mail</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Backend / Frontend</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alta</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pendente</t>
   </si>
   <si>
     <t xml:space="preserve">RNE1</t>
@@ -48,12 +66,21 @@
     <t xml:space="preserve">O e-mail do usuário deve ser único no sistema</t>
   </si>
   <si>
+    <t xml:space="preserve">Backend</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Banco de dados</t>
+  </si>
+  <si>
     <t xml:space="preserve">RNE2</t>
   </si>
   <si>
     <t xml:space="preserve">O usuário deve confirmar o e-mail para ativar a conta</t>
   </si>
   <si>
+    <t xml:space="preserve">RF2</t>
+  </si>
+  <si>
     <t xml:space="preserve">RNE3</t>
   </si>
   <si>
@@ -63,7 +90,13 @@
     <t xml:space="preserve">RNE4</t>
   </si>
   <si>
-    <t xml:space="preserve">O usuário terá opicionalmente os link's do github, e linkedin</t>
+    <t xml:space="preserve">O usuário terá opcionalmente links do GitHub e LinkedIn</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Frontend / Backend</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Baixa</t>
   </si>
   <si>
     <t xml:space="preserve">RNE5</t>
@@ -72,10 +105,16 @@
     <t xml:space="preserve">O usuário só pode editar, atualizar ou excluir seus próprios projetos</t>
   </si>
   <si>
+    <t xml:space="preserve">RF5, RF6</t>
+  </si>
+  <si>
     <t xml:space="preserve">RNE6</t>
   </si>
   <si>
-    <t xml:space="preserve">Níveis de usuários(Administrador, usuário comum)</t>
+    <t xml:space="preserve">Níveis de usuários (Administrador, usuário comum)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RF22</t>
   </si>
   <si>
     <t xml:space="preserve">RNE7</t>
@@ -84,28 +123,40 @@
     <t xml:space="preserve">Administradores podem remover conteúdos inadequados</t>
   </si>
   <si>
+    <t xml:space="preserve">RF20</t>
+  </si>
+  <si>
     <t xml:space="preserve">RNE8</t>
   </si>
   <si>
     <t xml:space="preserve">O usuário só pode editar/excluir seus próprios comentários</t>
   </si>
   <si>
+    <t xml:space="preserve">RF14, RF15</t>
+  </si>
+  <si>
     <t xml:space="preserve">RNE9</t>
   </si>
   <si>
-    <t xml:space="preserve">Os projetos podem ser privados, ou públicos</t>
+    <t xml:space="preserve">Os projetos podem ser privados ou públicos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RF8</t>
   </si>
   <si>
     <t xml:space="preserve">RNE10</t>
   </si>
   <si>
-    <t xml:space="preserve">Os projetos devem ter um fornecedor, nome, descrição, objetivo, link's e o tipo (nível)</t>
+    <t xml:space="preserve">Os projetos devem ter fornecedor, nome, descrição, objetivo, links e tipo (nível)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RF4</t>
   </si>
   <si>
     <t xml:space="preserve">RNE11</t>
   </si>
   <si>
-    <t xml:space="preserve">O projeto deve conter ao menos um link válido.</t>
+    <t xml:space="preserve">O projeto deve conter ao menos um link válido</t>
   </si>
   <si>
     <t xml:space="preserve">RNE12</t>
@@ -120,22 +171,31 @@
     <t xml:space="preserve">O tipo e nível do projeto devem seguir valores pré-definidos</t>
   </si>
   <si>
+    <t xml:space="preserve">RF10</t>
+  </si>
+  <si>
     <t xml:space="preserve">RNE14</t>
   </si>
   <si>
     <t xml:space="preserve">Projetos privados só podem ser vistos pelo autor</t>
   </si>
   <si>
+    <t xml:space="preserve">RF7</t>
+  </si>
+  <si>
     <t xml:space="preserve">RNE15</t>
   </si>
   <si>
     <t xml:space="preserve">Projetos públicos podem ser avaliados e comentados por outros usuários</t>
   </si>
   <si>
+    <t xml:space="preserve">RF13, RF17</t>
+  </si>
+  <si>
     <t xml:space="preserve">RNE16</t>
   </si>
   <si>
-    <t xml:space="preserve">Os links devem ser validados com URL válidas</t>
+    <t xml:space="preserve">Os links devem ser validados com URLs válidas</t>
   </si>
   <si>
     <t xml:space="preserve">RNE17</t>
@@ -144,6 +204,12 @@
     <t xml:space="preserve">Os projetos poderão ser atualizados</t>
   </si>
   <si>
+    <t xml:space="preserve">RF5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Média</t>
+  </si>
+  <si>
     <t xml:space="preserve">RNE18</t>
   </si>
   <si>
@@ -153,7 +219,10 @@
     <t xml:space="preserve">RNE19</t>
   </si>
   <si>
-    <t xml:space="preserve">Sistema deve possuir feedback, notas e visualizações para os projetos</t>
+    <t xml:space="preserve">O sistema deve possuir feedback, notas e visualizações para os projetos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RF17, RF19</t>
   </si>
   <si>
     <t xml:space="preserve">RNE20</t>
@@ -162,6 +231,9 @@
     <t xml:space="preserve">Um usuário pode avaliar um projeto somente uma vez</t>
   </si>
   <si>
+    <t xml:space="preserve">RF17</t>
+  </si>
+  <si>
     <t xml:space="preserve">RNE21</t>
   </si>
   <si>
@@ -174,64 +246,271 @@
     <t xml:space="preserve">A média da nota do projeto deve ser calculada automaticamente</t>
   </si>
   <si>
+    <t xml:space="preserve">RF18</t>
+  </si>
+  <si>
     <t xml:space="preserve">RNE23</t>
   </si>
   <si>
     <t xml:space="preserve">Comentários inadequados podem ser denunciados</t>
   </si>
   <si>
+    <t xml:space="preserve">RF16</t>
+  </si>
+  <si>
     <t xml:space="preserve">RNE24</t>
   </si>
   <si>
     <t xml:space="preserve">Comentários não podem ser vazios</t>
   </si>
   <si>
+    <t xml:space="preserve">RF13</t>
+  </si>
+  <si>
     <t xml:space="preserve">RNE25</t>
   </si>
   <si>
-    <t xml:space="preserve">Os comentários devem seguir as noemas de convivência do site</t>
+    <t xml:space="preserve">Comentários devem seguir normas de convivência do site</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Backend / Moderação</t>
   </si>
   <si>
     <t xml:space="preserve">RNE26</t>
   </si>
   <si>
-    <t xml:space="preserve">Comentários não devem conter tentativas de vender produtos</t>
+    <t xml:space="preserve">Comentários não devem conter tentativas de venda</t>
   </si>
   <si>
     <t xml:space="preserve">RNE27</t>
   </si>
   <si>
-    <t xml:space="preserve">O sistema deve possuir um buscador para os projetos</t>
+    <t xml:space="preserve">O sistema deve possuir um buscador para projetos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RF9</t>
   </si>
   <si>
     <t xml:space="preserve">RNE28</t>
   </si>
   <si>
-    <t xml:space="preserve">O buscador utilizará palavras chaves, do nome e do objetivo do projeto</t>
+    <t xml:space="preserve">O buscador utilizará palavras-chave do nome e objetivo do projeto</t>
   </si>
   <si>
     <t xml:space="preserve">RNE29</t>
   </si>
   <si>
-    <t xml:space="preserve">O buscador permitirá que seja buscado pelo o tipo, e o nível do projeto </t>
+    <t xml:space="preserve">O buscador permitirá busca por tipo e nível</t>
   </si>
   <si>
     <t xml:space="preserve">RNE30</t>
   </si>
   <si>
-    <t xml:space="preserve">A Busca deve ignorar letras maiúsculas/minúsculas</t>
+    <t xml:space="preserve">A busca deve ignorar letras maiúsculas/minúsculas</t>
   </si>
   <si>
     <t xml:space="preserve">RNE31</t>
   </si>
   <si>
-    <t xml:space="preserve">A busca deve permitir combinação de filtros (palavra-chave + nível + tipo)</t>
+    <t xml:space="preserve">A busca deve permitir combinação de filtros</t>
   </si>
   <si>
     <t xml:space="preserve">RNE32</t>
   </si>
   <si>
-    <t xml:space="preserve">Projetos mais bem avaliados devem ter prioridades nos resultados de busca</t>
+    <t xml:space="preserve">Projetos mais bem avaliados devem ter prioridade nos resultados</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RF11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RNF0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">O sistema deve responder às requisições do usuário em no máximo 2 segundos em condições normais</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Backend / Infraestrutura</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Servidor, rede</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RNF1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">O sistema deve suportar no mínimo 100 usuários simultâneos sem degradação significativa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Infraestrutura</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Servidor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RNF2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">O sistema deve garantir disponibilidade mínima de 95% do tempo (uptime)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hospedagem</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RNF3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">O sistema deve utilizar criptografia para armazenamento de senhas (hash seguro)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RNF4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">O sistema deve utilizar protocolo HTTPS para comunicação segura</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Infraestrutura / Backend</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Certificado SSL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RNF5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">O sistema deve validar e sanitizar todas as entradas de dados (proteção contra ataques)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Validação de entrada</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RNF6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">O sistema deve possuir controle de autenticação e autorização por nível de usuário</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RF22, RNE6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RNF7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">O sistema deve ser compatível com navegadores modernos (Chrome, Firefox, Edge)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Frontend</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Navegadores</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RNF8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">O sistema deve ser responsivo para dispositivos móveis e desktops</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CSS / Framework</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RNF9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">O sistema deve possuir interface intuitiva e de fácil uso</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Frontend / UX</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Design</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RNF10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">O sistema deve garantir persistência dos dados mesmo em falhas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RNF11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">O sistema deve realizar backup automático dos dados periodicamente</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RNF12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">O sistema deve registrar logs de atividades relevantes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RNF13</t>
+  </si>
+  <si>
+    <t xml:space="preserve">O sistema deve permitir manutenção sem perda de dados</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Versionamento</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RNF14</t>
+  </si>
+  <si>
+    <t xml:space="preserve">O código deve seguir boas práticas e padrões de desenvolvimento</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Desenvolvimento</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Equipe</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RNF15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">O sistema deve ser escalável para suportar crescimento de usuários</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Arquitetura do sistema</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RNF16</t>
+  </si>
+  <si>
+    <t xml:space="preserve">O tempo de carregamento das páginas deve ser inferior a 3 segundos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Otimização</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RNF17</t>
+  </si>
+  <si>
+    <t xml:space="preserve">O sistema deve tratar erros com mensagens claras ao usuário</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tratamento de exceções</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RNF18</t>
+  </si>
+  <si>
+    <t xml:space="preserve">O sistema deve proteger rotas contra acesso não autorizado</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RNF19</t>
+  </si>
+  <si>
+    <t xml:space="preserve">O sistema deve garantir integridade dos dados nas operações</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RNF20</t>
+  </si>
+  <si>
+    <t xml:space="preserve">O sistema deve permitir integração futura com APIs externas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Arquitetura modular</t>
   </si>
   <si>
     <t xml:space="preserve">RF0</t>
@@ -240,13 +519,16 @@
     <t xml:space="preserve">O sistema deve permitir o cadastro de usuários</t>
   </si>
   <si>
+    <t xml:space="preserve">RNE0, RNE1, RNE2, RNE3</t>
+  </si>
+  <si>
     <t xml:space="preserve">RF1</t>
   </si>
   <si>
     <t xml:space="preserve">O sistema deve permitir que o usuário faça login no sistema</t>
   </si>
   <si>
-    <t xml:space="preserve">RF2</t>
+    <t xml:space="preserve">RNE1, RNE2</t>
   </si>
   <si>
     <t xml:space="preserve">O sistema deve permitir a confirmação de e-mail para ativação da conta</t>
@@ -258,49 +540,46 @@
     <t xml:space="preserve">O sistema deve permitir a edição dos dados do usuário</t>
   </si>
   <si>
-    <t xml:space="preserve">RF4</t>
-  </si>
-  <si>
     <t xml:space="preserve">O sistema deve permitir o cadastro de projetos</t>
   </si>
   <si>
-    <t xml:space="preserve">RF5</t>
+    <t xml:space="preserve">RNE10, RNE11, RNE12, RNE13</t>
   </si>
   <si>
     <t xml:space="preserve">O sistema deve permitir a edição de projetos pelo autor</t>
   </si>
   <si>
+    <t xml:space="preserve">RNE5, RNE17</t>
+  </si>
+  <si>
     <t xml:space="preserve">RF6</t>
   </si>
   <si>
     <t xml:space="preserve">O sistema deve permitir a exclusão de projetos pelo autor</t>
   </si>
   <si>
-    <t xml:space="preserve">RF7</t>
-  </si>
-  <si>
     <t xml:space="preserve">O sistema deve permitir visualizar projetos públicos</t>
   </si>
   <si>
-    <t xml:space="preserve">RF8</t>
+    <t xml:space="preserve">RNE9, RNE15</t>
   </si>
   <si>
     <t xml:space="preserve">O sistema deve permitir definir projetos como públicos ou privados</t>
   </si>
   <si>
-    <t xml:space="preserve">RF9</t>
+    <t xml:space="preserve">RNE9, RNE14</t>
   </si>
   <si>
     <t xml:space="preserve">O sistema deve permitir buscar projetos por palavras-chave</t>
   </si>
   <si>
-    <t xml:space="preserve">RF10</t>
+    <t xml:space="preserve">RNE27, RNE28, RNE30</t>
   </si>
   <si>
     <t xml:space="preserve">O sistema deve permitir filtrar projetos por tipo e nível</t>
   </si>
   <si>
-    <t xml:space="preserve">RF11</t>
+    <t xml:space="preserve">RNE13, RNE29, RNE31</t>
   </si>
   <si>
     <t xml:space="preserve">O sistema deve permitir ordenar resultados de busca</t>
@@ -312,12 +591,12 @@
     <t xml:space="preserve">O sistema deve permitir visualizar detalhes de um projeto</t>
   </si>
   <si>
-    <t xml:space="preserve">RF13</t>
-  </si>
-  <si>
     <t xml:space="preserve">O sistema deve permitir adicionar comentários em projetos</t>
   </si>
   <si>
+    <t xml:space="preserve">RNE15, RNE24, RNE25, RNE26</t>
+  </si>
+  <si>
     <t xml:space="preserve">RF14</t>
   </si>
   <si>
@@ -330,19 +609,13 @@
     <t xml:space="preserve">O sistema deve permitir excluir comentários próprios</t>
   </si>
   <si>
-    <t xml:space="preserve">RF16</t>
-  </si>
-  <si>
     <t xml:space="preserve">O sistema deve permitir denunciar comentários</t>
   </si>
   <si>
-    <t xml:space="preserve">RF17</t>
-  </si>
-  <si>
     <t xml:space="preserve">O sistema deve permitir avaliar projetos</t>
   </si>
   <si>
-    <t xml:space="preserve">RF18</t>
+    <t xml:space="preserve">RNE20, RNE21</t>
   </si>
   <si>
     <t xml:space="preserve">O sistema deve calcular e exibir a média de avaliações dos projetos</t>
@@ -354,19 +627,16 @@
     <t xml:space="preserve">O sistema deve exibir número de visualizações dos projetos</t>
   </si>
   <si>
-    <t xml:space="preserve">RF20</t>
-  </si>
-  <si>
     <t xml:space="preserve">O sistema deve permitir que administradores removam conteúdos inadequados</t>
   </si>
   <si>
+    <t xml:space="preserve">RNE6, RNE7</t>
+  </si>
+  <si>
     <t xml:space="preserve">RF21</t>
   </si>
   <si>
     <t xml:space="preserve">O sistema deve permitir logout do usuário</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RF22</t>
   </si>
   <si>
     <t xml:space="preserve">O sistema deve restringir acesso a funcionalidades conforme tipo de usuário</t>
@@ -496,33 +766,29 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="7">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
@@ -824,12 +1090,14 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:F44"/>
-  <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="19.85" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.59375" defaultRowHeight="19.85" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="21.78"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="95.89"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="17.89"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="4" style="1" width="35.33"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="26.46"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="23.57"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="14.81"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="13.73"/>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="7" style="1" width="8.59"/>
   </cols>
   <sheetData>
@@ -846,305 +1114,671 @@
       <c r="D1" s="4" t="s">
         <v>3</v>
       </c>
+      <c r="E1" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>5</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="19.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="B2" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="C2" s="5"/>
-      <c r="D2" s="5"/>
+        <v>6</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="E2" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="F2" s="5" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="3" customFormat="false" ht="19.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="B3" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="C3" s="5"/>
-      <c r="D3" s="5"/>
+        <v>12</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="4" customFormat="false" ht="19.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="B4" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="C4" s="5"/>
-      <c r="D4" s="5"/>
+        <v>16</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="19.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="B5" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="C5" s="5"/>
-      <c r="D5" s="5"/>
+        <v>19</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="19.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="B6" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="C6" s="5"/>
-      <c r="D6" s="5"/>
+        <v>21</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="7" customFormat="false" ht="19.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="B7" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="C7" s="5"/>
-      <c r="D7" s="5"/>
+        <v>25</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="E7" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="F7" s="5" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="8" customFormat="false" ht="19.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="B8" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="C8" s="5"/>
-      <c r="D8" s="5"/>
+        <v>28</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="E8" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="F8" s="5" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="9" customFormat="false" ht="19.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="B9" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="C9" s="5"/>
-      <c r="D9" s="5"/>
+        <v>31</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="E9" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="F9" s="5" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="10" customFormat="false" ht="19.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="B10" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="C10" s="5"/>
-      <c r="D10" s="5"/>
+        <v>34</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D10" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="E10" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="F10" s="5" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="11" customFormat="false" ht="19.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="B11" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="C11" s="5"/>
-      <c r="D11" s="5"/>
+        <v>37</v>
+      </c>
+      <c r="B11" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="E11" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="F11" s="5" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="12" customFormat="false" ht="19.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="B12" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="C12" s="5"/>
-      <c r="D12" s="5"/>
-      <c r="E12" s="5"/>
-      <c r="F12" s="5"/>
+        <v>40</v>
+      </c>
+      <c r="B12" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D12" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="E12" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="F12" s="5" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="13" customFormat="false" ht="19.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="B13" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="C13" s="5"/>
-      <c r="D13" s="5"/>
-      <c r="E13" s="5"/>
-      <c r="F13" s="5"/>
+        <v>43</v>
+      </c>
+      <c r="B13" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="C13" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D13" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="E13" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="F13" s="5" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="14" customFormat="false" ht="19.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="B14" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="C14" s="5"/>
-      <c r="D14" s="5"/>
-      <c r="E14" s="5"/>
-      <c r="F14" s="5"/>
+        <v>45</v>
+      </c>
+      <c r="B14" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="C14" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D14" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="E14" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="F14" s="5" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="15" customFormat="false" ht="19.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="B15" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="C15" s="5"/>
-      <c r="D15" s="5"/>
+        <v>47</v>
+      </c>
+      <c r="B15" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="C15" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D15" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="E15" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="F15" s="5" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="16" customFormat="false" ht="19.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="5" t="s">
-        <v>32</v>
-      </c>
-      <c r="B16" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="C16" s="5"/>
-      <c r="D16" s="5"/>
+        <v>50</v>
+      </c>
+      <c r="B16" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="C16" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D16" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="E16" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="F16" s="5" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="17" customFormat="false" ht="19.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="B17" s="6" t="s">
-        <v>35</v>
+        <v>53</v>
+      </c>
+      <c r="B17" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="C17" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D17" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="E17" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="F17" s="5" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="19.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="B18" s="6" t="s">
-        <v>37</v>
+        <v>56</v>
+      </c>
+      <c r="B18" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="C18" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D18" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="E18" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="F18" s="5" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="19.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="5" t="s">
-        <v>38</v>
-      </c>
-      <c r="B19" s="6" t="s">
-        <v>39</v>
+        <v>58</v>
+      </c>
+      <c r="B19" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="C19" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D19" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="E19" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="F19" s="5" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="19.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="5" t="s">
-        <v>40</v>
-      </c>
-      <c r="B20" s="6" t="s">
-        <v>41</v>
+        <v>62</v>
+      </c>
+      <c r="B20" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="C20" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D20" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="E20" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="F20" s="5" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="19.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="B21" s="6" t="s">
-        <v>43</v>
+        <v>64</v>
+      </c>
+      <c r="B21" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="C21" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D21" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="E21" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="F21" s="5" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="19.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="5" t="s">
-        <v>44</v>
-      </c>
-      <c r="B22" s="6" t="s">
-        <v>45</v>
+        <v>67</v>
+      </c>
+      <c r="B22" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="C22" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D22" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="E22" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="F22" s="5" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="19.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="5" t="s">
-        <v>46</v>
-      </c>
-      <c r="B23" s="6" t="s">
-        <v>47</v>
+        <v>70</v>
+      </c>
+      <c r="B23" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="C23" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D23" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="E23" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="F23" s="5" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="19.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="5" t="s">
-        <v>48</v>
-      </c>
-      <c r="B24" s="6" t="s">
-        <v>49</v>
+        <v>72</v>
+      </c>
+      <c r="B24" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="C24" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D24" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="E24" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="F24" s="5" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="19.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="5" t="s">
-        <v>50</v>
-      </c>
-      <c r="B25" s="6" t="s">
-        <v>51</v>
+        <v>75</v>
+      </c>
+      <c r="B25" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="C25" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D25" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="E25" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="F25" s="5" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="19.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="B26" s="6" t="s">
-        <v>53</v>
+        <v>78</v>
+      </c>
+      <c r="B26" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="C26" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D26" s="5" t="s">
+        <v>80</v>
+      </c>
+      <c r="E26" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="F26" s="5" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="19.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="5" t="s">
-        <v>54</v>
-      </c>
-      <c r="B27" s="6" t="s">
-        <v>55</v>
+        <v>81</v>
+      </c>
+      <c r="B27" s="5" t="s">
+        <v>82</v>
+      </c>
+      <c r="C27" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="D27" s="5" t="s">
+        <v>80</v>
+      </c>
+      <c r="E27" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="F27" s="5" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="19.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="5" t="s">
-        <v>56</v>
-      </c>
-      <c r="B28" s="6" t="s">
-        <v>57</v>
+        <v>84</v>
+      </c>
+      <c r="B28" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="C28" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="D28" s="5" t="s">
+        <v>80</v>
+      </c>
+      <c r="E28" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="F28" s="5" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="19.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="5" t="s">
-        <v>58</v>
-      </c>
-      <c r="B29" s="6" t="s">
-        <v>59</v>
+        <v>86</v>
+      </c>
+      <c r="B29" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="C29" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D29" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="E29" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="F29" s="5" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="19.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="5" t="s">
-        <v>60</v>
-      </c>
-      <c r="B30" s="6" t="s">
-        <v>61</v>
+        <v>89</v>
+      </c>
+      <c r="B30" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="C30" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D30" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="E30" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="F30" s="5" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="19.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="5" t="s">
-        <v>62</v>
-      </c>
-      <c r="B31" s="6" t="s">
-        <v>63</v>
+        <v>91</v>
+      </c>
+      <c r="B31" s="5" t="s">
+        <v>92</v>
+      </c>
+      <c r="C31" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D31" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="E31" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="F31" s="5" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="19.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="5" t="s">
-        <v>64</v>
-      </c>
-      <c r="B32" s="6" t="s">
-        <v>65</v>
+        <v>93</v>
+      </c>
+      <c r="B32" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="C32" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D32" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="E32" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="F32" s="5" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="19.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="5" t="s">
-        <v>66</v>
-      </c>
-      <c r="B33" s="6" t="s">
-        <v>67</v>
+        <v>95</v>
+      </c>
+      <c r="B33" s="5" t="s">
+        <v>96</v>
+      </c>
+      <c r="C33" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D33" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="E33" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="F33" s="5" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="19.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="5" t="s">
-        <v>68</v>
-      </c>
-      <c r="B34" s="6" t="s">
-        <v>69</v>
+        <v>97</v>
+      </c>
+      <c r="B34" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="C34" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D34" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="E34" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="F34" s="5" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="19.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1205,17 +1839,20 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D24"/>
-  <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:F22"/>
+  <sheetFormatPr defaultColWidth="8.6015625" defaultRowHeight="19.85" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="17.63"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="94.88"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="16.96"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="14.1"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16376" style="0" width="10.16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="5" width="17.63"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="5" width="94.89"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="5" width="27"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="5" width="28.27"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="6" width="14.81"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="6" width="13.73"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16375" min="7" style="6" width="8.6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16376" style="5" width="10.16"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="22.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="19.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1228,236 +1865,432 @@
       <c r="D1" s="4" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="2" customFormat="false" ht="22.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="E1" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="19.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>70</v>
+        <v>100</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>71</v>
-      </c>
-      <c r="C2" s="5"/>
-      <c r="D2" s="5"/>
-    </row>
-    <row r="3" customFormat="false" ht="22.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>101</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>102</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="E2" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="F2" s="6" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="19.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="5" t="s">
-        <v>72</v>
+        <v>104</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>73</v>
-      </c>
-      <c r="C3" s="5"/>
-      <c r="D3" s="5"/>
-    </row>
-    <row r="4" customFormat="false" ht="22.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>105</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>106</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>107</v>
+      </c>
+      <c r="E3" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3" s="6" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="19.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
-        <v>74</v>
+        <v>108</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>75</v>
-      </c>
-      <c r="C4" s="5"/>
-      <c r="D4" s="5"/>
-    </row>
-    <row r="5" customFormat="false" ht="22.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>109</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>106</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="E4" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="F4" s="6" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="19.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>76</v>
+        <v>111</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>77</v>
-      </c>
-      <c r="C5" s="5"/>
-      <c r="D5" s="5"/>
-    </row>
-    <row r="6" customFormat="false" ht="22.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>112</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="E5" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="F5" s="6" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="19.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>78</v>
+        <v>113</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>79</v>
-      </c>
-      <c r="C6" s="5"/>
-      <c r="D6" s="5"/>
-    </row>
-    <row r="7" customFormat="false" ht="22.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>114</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>115</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>116</v>
+      </c>
+      <c r="E6" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="F6" s="6" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="19.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
-        <v>80</v>
+        <v>117</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>81</v>
-      </c>
-      <c r="C7" s="5"/>
-      <c r="D7" s="5"/>
-    </row>
-    <row r="8" customFormat="false" ht="22.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>118</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>119</v>
+      </c>
+      <c r="E7" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="F7" s="6" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="19.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
-        <v>82</v>
+        <v>120</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>83</v>
-      </c>
-      <c r="C8" s="5"/>
-      <c r="D8" s="5"/>
-    </row>
-    <row r="9" customFormat="false" ht="22.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>121</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>122</v>
+      </c>
+      <c r="E8" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="F8" s="6" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="19.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="s">
-        <v>84</v>
+        <v>123</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>85</v>
-      </c>
-      <c r="C9" s="5"/>
-      <c r="D9" s="5"/>
-    </row>
-    <row r="10" customFormat="false" ht="22.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>124</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>125</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>126</v>
+      </c>
+      <c r="E9" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="F9" s="6" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="19.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
-        <v>86</v>
+        <v>127</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>87</v>
-      </c>
-      <c r="C10" s="5"/>
-      <c r="D10" s="5"/>
-    </row>
-    <row r="11" customFormat="false" ht="22.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>128</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>125</v>
+      </c>
+      <c r="D10" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="E10" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="F10" s="6" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="19.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="s">
-        <v>88</v>
+        <v>130</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>89</v>
-      </c>
-      <c r="C11" s="5"/>
-      <c r="D11" s="5"/>
-    </row>
-    <row r="12" customFormat="false" ht="22.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>131</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>132</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>133</v>
+      </c>
+      <c r="E11" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="F11" s="6" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="19.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="5" t="s">
-        <v>90</v>
+        <v>134</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>91</v>
-      </c>
-      <c r="C12" s="5"/>
-      <c r="D12" s="5"/>
-    </row>
-    <row r="13" customFormat="false" ht="22.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>135</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D12" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="E12" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="F12" s="6" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="19.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="5" t="s">
-        <v>92</v>
+        <v>136</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>93</v>
-      </c>
-      <c r="C13" s="5"/>
-      <c r="D13" s="5"/>
-    </row>
-    <row r="14" customFormat="false" ht="22.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>137</v>
+      </c>
+      <c r="C13" s="5" t="s">
+        <v>106</v>
+      </c>
+      <c r="D13" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="E13" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="F13" s="6" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="19.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="5" t="s">
-        <v>94</v>
+        <v>138</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>95</v>
-      </c>
-      <c r="C14" s="5"/>
-      <c r="D14" s="5"/>
-    </row>
-    <row r="15" customFormat="false" ht="22.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>139</v>
+      </c>
+      <c r="C14" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D14" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="E14" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="F14" s="6" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="19.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="5" t="s">
-        <v>96</v>
+        <v>140</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>97</v>
-      </c>
-      <c r="C15" s="5"/>
-      <c r="D15" s="5"/>
-    </row>
-    <row r="16" customFormat="false" ht="22.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>141</v>
+      </c>
+      <c r="C15" s="5" t="s">
+        <v>102</v>
+      </c>
+      <c r="D15" s="5" t="s">
+        <v>142</v>
+      </c>
+      <c r="E15" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="F15" s="6" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="19.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="5" t="s">
-        <v>98</v>
+        <v>143</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>99</v>
-      </c>
-      <c r="C16" s="5"/>
-      <c r="D16" s="5"/>
-    </row>
-    <row r="17" customFormat="false" ht="22.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>144</v>
+      </c>
+      <c r="C16" s="5" t="s">
+        <v>145</v>
+      </c>
+      <c r="D16" s="5" t="s">
+        <v>146</v>
+      </c>
+      <c r="E16" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="F16" s="6" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="19.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="5" t="s">
-        <v>100</v>
+        <v>147</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>101</v>
-      </c>
-      <c r="C17" s="5"/>
-      <c r="D17" s="5"/>
-    </row>
-    <row r="18" customFormat="false" ht="22.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>148</v>
+      </c>
+      <c r="C17" s="5" t="s">
+        <v>106</v>
+      </c>
+      <c r="D17" s="5" t="s">
+        <v>149</v>
+      </c>
+      <c r="E17" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="F17" s="6" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="19.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="5" t="s">
-        <v>102</v>
+        <v>150</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>103</v>
-      </c>
-      <c r="C18" s="5"/>
-      <c r="D18" s="5"/>
-    </row>
-    <row r="19" customFormat="false" ht="22.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>151</v>
+      </c>
+      <c r="C18" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="D18" s="5" t="s">
+        <v>152</v>
+      </c>
+      <c r="E18" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="F18" s="6" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="19.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="5" t="s">
-        <v>104</v>
+        <v>153</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>105</v>
-      </c>
-      <c r="C19" s="5"/>
-      <c r="D19" s="5"/>
-    </row>
-    <row r="20" customFormat="false" ht="22.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>154</v>
+      </c>
+      <c r="C19" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="D19" s="5" t="s">
+        <v>155</v>
+      </c>
+      <c r="E19" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="F19" s="6" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="19.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="5" t="s">
-        <v>106</v>
+        <v>156</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>107</v>
-      </c>
-      <c r="C20" s="5"/>
-      <c r="D20" s="5"/>
-    </row>
-    <row r="21" customFormat="false" ht="22.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>157</v>
+      </c>
+      <c r="C20" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D20" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="E20" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="F20" s="6" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="19.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="5" t="s">
-        <v>108</v>
+        <v>158</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>109</v>
-      </c>
-      <c r="C21" s="5"/>
-      <c r="D21" s="5"/>
-    </row>
-    <row r="22" customFormat="false" ht="22.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>159</v>
+      </c>
+      <c r="C21" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D21" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="E21" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="F21" s="6" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="19.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="5" t="s">
-        <v>110</v>
+        <v>160</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>111</v>
-      </c>
-      <c r="C22" s="5"/>
-      <c r="D22" s="5"/>
-    </row>
-    <row r="23" customFormat="false" ht="22.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="5" t="s">
-        <v>112</v>
-      </c>
-      <c r="B23" s="5" t="s">
-        <v>113</v>
-      </c>
-      <c r="C23" s="5"/>
-      <c r="D23" s="5"/>
-    </row>
-    <row r="24" customFormat="false" ht="22.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="5" t="s">
-        <v>114</v>
-      </c>
-      <c r="B24" s="5" t="s">
-        <v>115</v>
-      </c>
-      <c r="C24" s="5"/>
-      <c r="D24" s="5"/>
+        <v>161</v>
+      </c>
+      <c r="C22" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D22" s="5" t="s">
+        <v>162</v>
+      </c>
+      <c r="E22" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="F22" s="6" t="s">
+        <v>11</v>
+      </c>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -1475,18 +2308,20 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:XFD24"/>
-  <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="22.7" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:H24"/>
+  <sheetFormatPr defaultColWidth="8.59375" defaultRowHeight="19.85" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="5" width="17.63"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="5" width="92.63"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="5" width="27.31"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="5" width="24.45"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16379" min="5" style="5" width="8.59"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="5" width="24.46"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="5" width="14.81"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="5" width="13.73"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16379" min="7" style="5" width="8.59"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16380" style="5" width="10.16"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="22.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="19.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1499,193 +2334,472 @@
       <c r="D1" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="XFA1" s="7"/>
-      <c r="XFB1" s="7"/>
-      <c r="XFC1" s="7"/>
-      <c r="XFD1" s="7"/>
-    </row>
-    <row r="2" customFormat="false" ht="22.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="E1" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="19.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>70</v>
+        <v>163</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="3" customFormat="false" ht="22.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>164</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>165</v>
+      </c>
+      <c r="E2" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="F2" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="19.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="5" t="s">
-        <v>72</v>
+        <v>166</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="22.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>167</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>168</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="H3" s="0"/>
+    </row>
+    <row r="4" customFormat="false" ht="19.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
-        <v>74</v>
+        <v>18</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="22.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>169</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="19.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>76</v>
+        <v>170</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="22.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>171</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="19.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>78</v>
+        <v>42</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="22.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>172</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>173</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="19.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="22.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>174</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>175</v>
+      </c>
+      <c r="E7" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="F7" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="19.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
-        <v>82</v>
+        <v>176</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="22.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>177</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="E8" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="F8" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="19.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="s">
-        <v>84</v>
+        <v>52</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="22.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>178</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>179</v>
+      </c>
+      <c r="E9" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="F9" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="19.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
-        <v>86</v>
+        <v>39</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="22.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>180</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D10" s="5" t="s">
+        <v>181</v>
+      </c>
+      <c r="E10" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="F10" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="19.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="s">
         <v>88</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="22.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>182</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>183</v>
+      </c>
+      <c r="E11" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="F11" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="19.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="5" t="s">
-        <v>90</v>
+        <v>49</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="22.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>184</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D12" s="5" t="s">
+        <v>185</v>
+      </c>
+      <c r="E12" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="F12" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="19.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="5" t="s">
-        <v>92</v>
+        <v>99</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="22.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>186</v>
+      </c>
+      <c r="C13" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D13" s="5" t="s">
+        <v>97</v>
+      </c>
+      <c r="E13" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="F13" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="19.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="5" t="s">
-        <v>94</v>
+        <v>187</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="22.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>188</v>
+      </c>
+      <c r="C14" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="D14" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="E14" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="F14" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="19.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="5" t="s">
-        <v>96</v>
+        <v>80</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="22.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>189</v>
+      </c>
+      <c r="C15" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D15" s="5" t="s">
+        <v>190</v>
+      </c>
+      <c r="E15" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="F15" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="19.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="5" t="s">
-        <v>98</v>
+        <v>191</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="22.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>192</v>
+      </c>
+      <c r="C16" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D16" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="E16" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="F16" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="19.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="5" t="s">
-        <v>100</v>
+        <v>193</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="22.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>194</v>
+      </c>
+      <c r="C17" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D17" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="E17" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="F17" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="19.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="5" t="s">
-        <v>102</v>
+        <v>77</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="22.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>195</v>
+      </c>
+      <c r="C18" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D18" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="E18" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="F18" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="19.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="5" t="s">
-        <v>104</v>
+        <v>69</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="22.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>196</v>
+      </c>
+      <c r="C19" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D19" s="5" t="s">
+        <v>197</v>
+      </c>
+      <c r="E19" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="F19" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="19.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="5" t="s">
-        <v>106</v>
+        <v>74</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="22.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>198</v>
+      </c>
+      <c r="C20" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D20" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="E20" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="F20" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="19.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="5" t="s">
-        <v>108</v>
+        <v>199</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="22.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>200</v>
+      </c>
+      <c r="C21" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D21" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="E21" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="F21" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="19.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="5" t="s">
-        <v>110</v>
+        <v>33</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="22.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>201</v>
+      </c>
+      <c r="C22" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D22" s="5" t="s">
+        <v>202</v>
+      </c>
+      <c r="E22" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="F22" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="19.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="5" t="s">
-        <v>112</v>
+        <v>203</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="22.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>204</v>
+      </c>
+      <c r="C23" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D23" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="E23" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="F23" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="19.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="5" t="s">
-        <v>114</v>
+        <v>30</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>115</v>
+        <v>205</v>
+      </c>
+      <c r="C24" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D24" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="E24" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="F24" s="5" t="s">
+        <v>11</v>
       </c>
     </row>
   </sheetData>

</xml_diff>